<commit_message>
update: final finish project
</commit_message>
<xml_diff>
--- a/ket_qua/14_Bang_phan_chia_luong/Bang_phan_chia_luong.xlsx
+++ b/ket_qua/14_Bang_phan_chia_luong/Bang_phan_chia_luong.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2381" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2383" uniqueCount="322">
   <si>
     <t xml:space="preserve">Bảng phân chia lương</t>
   </si>
@@ -35,7 +35,7 @@
     <t xml:space="preserve">Xây dựng và triển khai hệ thống website bán hàng trực tuyến (Web Selling Site System)</t>
   </si>
   <si>
-    <t xml:space="preserve">Nhóm PM_26I_02, PM_26I_02</t>
+    <t xml:space="preserve">Nhóm PM_26I_02</t>
   </si>
   <si>
     <t xml:space="preserve">Số liệu tính đến ngày 12/08/2027. Cách trả lương do nhóm khai báo: trả theo công sức (MD công việc).</t>
@@ -47,7 +47,7 @@
     <t xml:space="preserve">1. Công sức thực tế theo nhật ký công việc (sheet Nhat_ky), mỗi dòng là MD của một thành viên cho một gói WBS trong một ngày.</t>
   </si>
   <si>
-    <t xml:space="preserve">2. Ngày huy động theo kế hoạch huy động của master schedule (sheet Huy_dong), cùng nguồn với cost estimate, tính đến ngày trên.</t>
+    <t xml:space="preserve">2. Ngày huy động theo kế hoạch huy động của master schedule (sheet Huy_dong), cùng nguồn với cost estimate, tính đến ngày trên, cộng huy động bổ sung thực tế theo nhu cầu 13 MD theo dau_vao/thuc_te/huy_dong_bo_sung.json.</t>
   </si>
   <si>
     <t xml:space="preserve">3. Đơn giá ngày của vai trò bằng lương tham chiếu tháng chia số ngày làm việc mỗi tháng (sheet Tham_so).</t>
@@ -62,7 +62,7 @@
     <t xml:space="preserve">6. Ngày sẵn sàng không ghi công bằng ngày huy động trừ MD thực tế, trình bày riêng để đối chiếu, không dùng để trừ lương.</t>
   </si>
   <si>
-    <t xml:space="preserve">7. Bảng đối chiếu MD kế hoạch theo master schedule, khoản A và chi phí lương theo huy động của cost estimate (sheet Doi_chieu).</t>
+    <t xml:space="preserve">7. Bảng đối chiếu MD kế hoạch theo master schedule, khoản A và chi phí lương kế hoạch của cost estimate theo cùng cách trả lương (MD công việc, sheet Doi_chieu).</t>
   </si>
   <si>
     <t xml:space="preserve">8. Số liệu thực tế trong bảng là số liệu mô phỏng. Số liệu mô phỏng: dữ liệu thực tế trong dau_vao/thuc_te/ do script qlda-mo-phong/scripts/mo_phong_sprint.py sinh từ kịch bản biến cố từng sprint (lam_viec/mo_phong/kich_ban_S&lt;n&gt;.json) theo kế hoạch đã duyệt hiện hành, không phải số liệu đo được của dự án thật.</t>
@@ -1712,7 +1712,7 @@
         <v>66.33</v>
       </c>
       <c r="G2" s="8" t="n">
-        <f aca="false">SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,B2)</f>
+        <f aca="false">SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,B2)</f>
         <v>86</v>
       </c>
       <c r="H2" s="8" t="n">
@@ -1781,8 +1781,8 @@
         <v>50</v>
       </c>
       <c r="G3" s="8" t="n">
-        <f aca="false">SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,B3)</f>
-        <v>69</v>
+        <f aca="false">SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,B3)</f>
+        <v>70.5</v>
       </c>
       <c r="H3" s="8" t="n">
         <f aca="false">SUMIFS(Nhat_ky!$E$2:$E$989,Nhat_ky!$C$2:$C$989,B3)</f>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="I3" s="9" t="n">
         <f aca="false">G3-H3</f>
-        <v>18.75</v>
+        <v>20.25</v>
       </c>
       <c r="J3" s="9" t="n">
         <f aca="false">H3-F3</f>
@@ -1850,8 +1850,8 @@
         <v>58</v>
       </c>
       <c r="G4" s="8" t="n">
-        <f aca="false">SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,B4)</f>
-        <v>71</v>
+        <f aca="false">SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,B4)</f>
+        <v>72</v>
       </c>
       <c r="H4" s="8" t="n">
         <f aca="false">SUMIFS(Nhat_ky!$E$2:$E$989,Nhat_ky!$C$2:$C$989,B4)</f>
@@ -1859,7 +1859,7 @@
       </c>
       <c r="I4" s="9" t="n">
         <f aca="false">G4-H4</f>
-        <v>13.5</v>
+        <v>14.5</v>
       </c>
       <c r="J4" s="9" t="n">
         <f aca="false">H4-F4</f>
@@ -1919,7 +1919,7 @@
         <v>66.5</v>
       </c>
       <c r="G5" s="8" t="n">
-        <f aca="false">SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,B5)</f>
+        <f aca="false">SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,B5)</f>
         <v>76</v>
       </c>
       <c r="H5" s="8" t="n">
@@ -1988,8 +1988,8 @@
         <v>72.5</v>
       </c>
       <c r="G6" s="8" t="n">
-        <f aca="false">SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,B6)</f>
-        <v>83</v>
+        <f aca="false">SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,B6)</f>
+        <v>84</v>
       </c>
       <c r="H6" s="8" t="n">
         <f aca="false">SUMIFS(Nhat_ky!$E$2:$E$989,Nhat_ky!$C$2:$C$989,B6)</f>
@@ -1997,7 +1997,7 @@
       </c>
       <c r="I6" s="9" t="n">
         <f aca="false">G6-H6</f>
-        <v>9.75</v>
+        <v>10.75</v>
       </c>
       <c r="J6" s="9" t="n">
         <f aca="false">H6-F6</f>
@@ -2057,7 +2057,7 @@
         <v>70.67</v>
       </c>
       <c r="G7" s="8" t="n">
-        <f aca="false">SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,B7)</f>
+        <f aca="false">SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,B7)</f>
         <v>80</v>
       </c>
       <c r="H7" s="8" t="n">
@@ -2126,8 +2126,8 @@
         <v>67.5</v>
       </c>
       <c r="G8" s="8" t="n">
-        <f aca="false">SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,B8)</f>
-        <v>85</v>
+        <f aca="false">SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,B8)</f>
+        <v>86</v>
       </c>
       <c r="H8" s="8" t="n">
         <f aca="false">SUMIFS(Nhat_ky!$E$2:$E$989,Nhat_ky!$C$2:$C$989,B8)</f>
@@ -2135,7 +2135,7 @@
       </c>
       <c r="I8" s="9" t="n">
         <f aca="false">G8-H8</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J8" s="9" t="n">
         <f aca="false">H8-F8</f>
@@ -2195,8 +2195,8 @@
         <v>64</v>
       </c>
       <c r="G9" s="8" t="n">
-        <f aca="false">SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,B9)</f>
-        <v>77</v>
+        <f aca="false">SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,B9)</f>
+        <v>78</v>
       </c>
       <c r="H9" s="8" t="n">
         <f aca="false">SUMIFS(Nhat_ky!$E$2:$E$989,Nhat_ky!$C$2:$C$989,B9)</f>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="I9" s="9" t="n">
         <f aca="false">G9-H9</f>
-        <v>12.75</v>
+        <v>13.75</v>
       </c>
       <c r="J9" s="9" t="n">
         <f aca="false">H9-F9</f>
@@ -2264,7 +2264,7 @@
         <v>59.5</v>
       </c>
       <c r="G10" s="8" t="n">
-        <f aca="false">SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,B10)</f>
+        <f aca="false">SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,B10)</f>
         <v>86</v>
       </c>
       <c r="H10" s="8" t="n">
@@ -2333,8 +2333,8 @@
         <v>49.5</v>
       </c>
       <c r="G11" s="8" t="n">
-        <f aca="false">SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,B11)</f>
-        <v>70</v>
+        <f aca="false">SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,B11)</f>
+        <v>72</v>
       </c>
       <c r="H11" s="8" t="n">
         <f aca="false">SUMIFS(Nhat_ky!$E$2:$E$989,Nhat_ky!$C$2:$C$989,B11)</f>
@@ -2342,7 +2342,7 @@
       </c>
       <c r="I11" s="9" t="n">
         <f aca="false">G11-H11</f>
-        <v>20.25</v>
+        <v>22.25</v>
       </c>
       <c r="J11" s="9" t="n">
         <f aca="false">H11-F11</f>
@@ -2402,8 +2402,8 @@
         <v>50</v>
       </c>
       <c r="G12" s="8" t="n">
-        <f aca="false">SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,B12)</f>
-        <v>63</v>
+        <f aca="false">SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,B12)</f>
+        <v>66</v>
       </c>
       <c r="H12" s="8" t="n">
         <f aca="false">SUMIFS(Nhat_ky!$E$2:$E$989,Nhat_ky!$C$2:$C$989,B12)</f>
@@ -2411,7 +2411,7 @@
       </c>
       <c r="I12" s="9" t="n">
         <f aca="false">G12-H12</f>
-        <v>13.75</v>
+        <v>16.75</v>
       </c>
       <c r="J12" s="9" t="n">
         <f aca="false">H12-F12</f>
@@ -2471,8 +2471,8 @@
         <v>58.5</v>
       </c>
       <c r="G13" s="8" t="n">
-        <f aca="false">SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,B13)</f>
-        <v>62</v>
+        <f aca="false">SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,B13)</f>
+        <v>64.5</v>
       </c>
       <c r="H13" s="8" t="n">
         <f aca="false">SUMIFS(Nhat_ky!$E$2:$E$989,Nhat_ky!$C$2:$C$989,B13)</f>
@@ -2480,7 +2480,7 @@
       </c>
       <c r="I13" s="9" t="n">
         <f aca="false">G13-H13</f>
-        <v>3.25</v>
+        <v>5.75</v>
       </c>
       <c r="J13" s="9" t="n">
         <f aca="false">H13-F13</f>
@@ -2530,7 +2530,7 @@
       </c>
       <c r="G14" s="14" t="n">
         <f aca="false">SUM(G2:G13)</f>
-        <v>908</v>
+        <v>921</v>
       </c>
       <c r="H14" s="14" t="n">
         <f aca="false">SUM(H2:H13)</f>
@@ -2538,7 +2538,7 @@
       </c>
       <c r="I14" s="14" t="n">
         <f aca="false">SUM(I2:I13)</f>
-        <v>171.25</v>
+        <v>184.25</v>
       </c>
       <c r="J14" s="14" t="n">
         <f aca="false">SUM(J2:J13)</f>
@@ -2736,43 +2736,43 @@
         <v>67.25</v>
       </c>
       <c r="N2" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",C2,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A2,Huy_dong!$B$2:$B$99,"S1"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A2,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",C2,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A2,Huy_dong!$B$2:$B$100,"S1"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A2,Bang_luong!$B$2:$B$13,0))</f>
         <v>23181818.1818182</v>
       </c>
       <c r="O2" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",D2,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A2,Huy_dong!$B$2:$B$99,"S2"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A2,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",D2,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A2,Huy_dong!$B$2:$B$100,"S2"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A2,Bang_luong!$B$2:$B$13,0))</f>
         <v>23181818.1818182</v>
       </c>
       <c r="P2" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",E2,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A2,Huy_dong!$B$2:$B$99,"S3"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A2,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",E2,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A2,Huy_dong!$B$2:$B$100,"S3"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A2,Bang_luong!$B$2:$B$13,0))</f>
         <v>29556818.1818182</v>
       </c>
       <c r="Q2" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",F2,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A2,Huy_dong!$B$2:$B$99,"S4"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A2,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",F2,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A2,Huy_dong!$B$2:$B$100,"S4"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A2,Bang_luong!$B$2:$B$13,0))</f>
         <v>23181818.1818182</v>
       </c>
       <c r="R2" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",G2,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A2,Huy_dong!$B$2:$B$99,"S5"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A2,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",G2,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A2,Huy_dong!$B$2:$B$100,"S5"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A2,Bang_luong!$B$2:$B$13,0))</f>
         <v>6954545.45454546</v>
       </c>
       <c r="S2" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",H2,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A2,Huy_dong!$B$2:$B$99,"S6"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A2,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",H2,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A2,Huy_dong!$B$2:$B$100,"S6"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A2,Bang_luong!$B$2:$B$13,0))</f>
         <v>10431818.1818182</v>
       </c>
       <c r="T2" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",I2,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A2,Huy_dong!$B$2:$B$99,"S7"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A2,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",I2,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A2,Huy_dong!$B$2:$B$100,"S7"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A2,Bang_luong!$B$2:$B$13,0))</f>
         <v>12170454.5454545</v>
       </c>
       <c r="U2" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",J2,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A2,Huy_dong!$B$2:$B$99,"S8"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A2,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",J2,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A2,Huy_dong!$B$2:$B$100,"S8"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A2,Bang_luong!$B$2:$B$13,0))</f>
         <v>15647727.2727273</v>
       </c>
       <c r="V2" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",K2,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A2,Huy_dong!$B$2:$B$99,"S9"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A2,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",K2,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A2,Huy_dong!$B$2:$B$100,"S9"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A2,Bang_luong!$B$2:$B$13,0))</f>
         <v>6954545.45454546</v>
       </c>
       <c r="W2" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",L2,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A2,Huy_dong!$B$2:$B$99,"KT"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A2,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",L2,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A2,Huy_dong!$B$2:$B$100,"KT"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A2,Bang_luong!$B$2:$B$13,0))</f>
         <v>4636363.63636364</v>
       </c>
       <c r="X2" s="12" t="n">
@@ -2832,43 +2832,43 @@
         <v>50.25</v>
       </c>
       <c r="N3" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",C3,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A3,Huy_dong!$B$2:$B$99,"S1"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A3,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",C3,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A3,Huy_dong!$B$2:$B$100,"S1"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A3,Bang_luong!$B$2:$B$13,0))</f>
         <v>5454545.45454545</v>
       </c>
       <c r="O3" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",D3,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A3,Huy_dong!$B$2:$B$99,"S2"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A3,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",D3,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A3,Huy_dong!$B$2:$B$100,"S2"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A3,Bang_luong!$B$2:$B$13,0))</f>
         <v>6818181.81818182</v>
       </c>
       <c r="P3" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",E3,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A3,Huy_dong!$B$2:$B$99,"S3"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A3,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",E3,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A3,Huy_dong!$B$2:$B$100,"S3"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A3,Bang_luong!$B$2:$B$13,0))</f>
         <v>9545454.54545455</v>
       </c>
       <c r="Q3" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",F3,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A3,Huy_dong!$B$2:$B$99,"S4"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A3,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",F3,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A3,Huy_dong!$B$2:$B$100,"S4"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A3,Bang_luong!$B$2:$B$13,0))</f>
         <v>13636363.6363636</v>
       </c>
       <c r="R3" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",G3,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A3,Huy_dong!$B$2:$B$99,"S5"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A3,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",G3,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A3,Huy_dong!$B$2:$B$100,"S5"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A3,Bang_luong!$B$2:$B$13,0))</f>
         <v>13636363.6363636</v>
       </c>
       <c r="S3" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",H3,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A3,Huy_dong!$B$2:$B$99,"S6"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A3,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",H3,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A3,Huy_dong!$B$2:$B$100,"S6"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A3,Bang_luong!$B$2:$B$13,0))</f>
         <v>11250000</v>
       </c>
       <c r="T3" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",I3,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A3,Huy_dong!$B$2:$B$99,"S7"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A3,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",I3,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A3,Huy_dong!$B$2:$B$100,"S7"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A3,Bang_luong!$B$2:$B$13,0))</f>
         <v>0</v>
       </c>
       <c r="U3" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",J3,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A3,Huy_dong!$B$2:$B$99,"S8"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A3,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",J3,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A3,Huy_dong!$B$2:$B$100,"S8"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A3,Bang_luong!$B$2:$B$13,0))</f>
         <v>1363636.36363636</v>
       </c>
       <c r="V3" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",K3,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A3,Huy_dong!$B$2:$B$99,"S9"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A3,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",K3,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A3,Huy_dong!$B$2:$B$100,"S9"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A3,Bang_luong!$B$2:$B$13,0))</f>
         <v>6818181.81818182</v>
       </c>
       <c r="W3" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",L3,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A3,Huy_dong!$B$2:$B$99,"KT"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A3,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",L3,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A3,Huy_dong!$B$2:$B$100,"KT"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A3,Bang_luong!$B$2:$B$13,0))</f>
         <v>0</v>
       </c>
       <c r="X3" s="12" t="n">
@@ -2928,43 +2928,43 @@
         <v>57.5</v>
       </c>
       <c r="N4" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",C4,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A4,Huy_dong!$B$2:$B$99,"S1"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A4,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",C4,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A4,Huy_dong!$B$2:$B$100,"S1"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A4,Bang_luong!$B$2:$B$13,0))</f>
         <v>10818181.8181818</v>
       </c>
       <c r="O4" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",D4,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A4,Huy_dong!$B$2:$B$99,"S2"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A4,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",D4,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A4,Huy_dong!$B$2:$B$100,"S2"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A4,Bang_luong!$B$2:$B$13,0))</f>
         <v>12727272.7272727</v>
       </c>
       <c r="P4" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",E4,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A4,Huy_dong!$B$2:$B$99,"S3"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A4,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",E4,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A4,Huy_dong!$B$2:$B$100,"S3"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A4,Bang_luong!$B$2:$B$13,0))</f>
         <v>14000000</v>
       </c>
       <c r="Q4" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",F4,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A4,Huy_dong!$B$2:$B$99,"S4"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A4,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",F4,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A4,Huy_dong!$B$2:$B$100,"S4"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A4,Bang_luong!$B$2:$B$13,0))</f>
         <v>12409090.9090909</v>
       </c>
       <c r="R4" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",G4,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A4,Huy_dong!$B$2:$B$99,"S5"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A4,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",G4,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A4,Huy_dong!$B$2:$B$100,"S5"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A4,Bang_luong!$B$2:$B$13,0))</f>
         <v>7954545.45454545</v>
       </c>
       <c r="S4" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",H4,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A4,Huy_dong!$B$2:$B$99,"S6"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A4,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",H4,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A4,Huy_dong!$B$2:$B$100,"S6"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A4,Bang_luong!$B$2:$B$13,0))</f>
         <v>6045454.54545455</v>
       </c>
       <c r="T4" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",I4,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A4,Huy_dong!$B$2:$B$99,"S7"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A4,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",I4,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A4,Huy_dong!$B$2:$B$100,"S7"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A4,Bang_luong!$B$2:$B$13,0))</f>
         <v>0</v>
       </c>
       <c r="U4" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",J4,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A4,Huy_dong!$B$2:$B$99,"S8"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A4,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",J4,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A4,Huy_dong!$B$2:$B$100,"S8"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A4,Bang_luong!$B$2:$B$13,0))</f>
         <v>4136363.63636364</v>
       </c>
       <c r="V4" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",K4,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A4,Huy_dong!$B$2:$B$99,"S9"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A4,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",K4,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A4,Huy_dong!$B$2:$B$100,"S9"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A4,Bang_luong!$B$2:$B$13,0))</f>
         <v>5090909.09090909</v>
       </c>
       <c r="W4" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",L4,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A4,Huy_dong!$B$2:$B$99,"KT"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A4,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",L4,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A4,Huy_dong!$B$2:$B$100,"KT"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A4,Bang_luong!$B$2:$B$13,0))</f>
         <v>0</v>
       </c>
       <c r="X4" s="12" t="n">
@@ -3024,43 +3024,43 @@
         <v>67.5</v>
       </c>
       <c r="N5" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",C5,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A5,Huy_dong!$B$2:$B$99,"S1"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A5,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",C5,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A5,Huy_dong!$B$2:$B$100,"S1"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A5,Bang_luong!$B$2:$B$13,0))</f>
         <v>8181818.18181818</v>
       </c>
       <c r="O5" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",D5,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A5,Huy_dong!$B$2:$B$99,"S2"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A5,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",D5,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A5,Huy_dong!$B$2:$B$100,"S2"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A5,Bang_luong!$B$2:$B$13,0))</f>
         <v>11931818.1818182</v>
       </c>
       <c r="P5" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",E5,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A5,Huy_dong!$B$2:$B$99,"S3"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A5,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",E5,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A5,Huy_dong!$B$2:$B$100,"S3"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A5,Bang_luong!$B$2:$B$13,0))</f>
         <v>17727272.7272727</v>
       </c>
       <c r="Q5" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",F5,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A5,Huy_dong!$B$2:$B$99,"S4"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A5,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",F5,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A5,Huy_dong!$B$2:$B$100,"S4"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A5,Bang_luong!$B$2:$B$13,0))</f>
         <v>13636363.6363636</v>
       </c>
       <c r="R5" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",G5,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A5,Huy_dong!$B$2:$B$99,"S5"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A5,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",G5,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A5,Huy_dong!$B$2:$B$100,"S5"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A5,Bang_luong!$B$2:$B$13,0))</f>
         <v>10568181.8181818</v>
       </c>
       <c r="S5" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",H5,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A5,Huy_dong!$B$2:$B$99,"S6"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A5,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",H5,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A5,Huy_dong!$B$2:$B$100,"S6"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A5,Bang_luong!$B$2:$B$13,0))</f>
         <v>13636363.6363636</v>
       </c>
       <c r="T5" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",I5,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A5,Huy_dong!$B$2:$B$99,"S7"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A5,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",I5,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A5,Huy_dong!$B$2:$B$100,"S7"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A5,Bang_luong!$B$2:$B$13,0))</f>
         <v>4090909.09090909</v>
       </c>
       <c r="U5" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",J5,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A5,Huy_dong!$B$2:$B$99,"S8"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A5,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",J5,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A5,Huy_dong!$B$2:$B$100,"S8"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A5,Bang_luong!$B$2:$B$13,0))</f>
         <v>0</v>
       </c>
       <c r="V5" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",K5,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A5,Huy_dong!$B$2:$B$99,"S9"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A5,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",K5,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A5,Huy_dong!$B$2:$B$100,"S9"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A5,Bang_luong!$B$2:$B$13,0))</f>
         <v>12272727.2727273</v>
       </c>
       <c r="W5" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",L5,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A5,Huy_dong!$B$2:$B$99,"KT"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A5,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",L5,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A5,Huy_dong!$B$2:$B$100,"KT"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A5,Bang_luong!$B$2:$B$13,0))</f>
         <v>0</v>
       </c>
       <c r="X5" s="12" t="n">
@@ -3120,43 +3120,43 @@
         <v>73.25</v>
       </c>
       <c r="N6" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",C6,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A6,Huy_dong!$B$2:$B$99,"S1"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A6,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",C6,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A6,Huy_dong!$B$2:$B$100,"S1"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A6,Bang_luong!$B$2:$B$13,0))</f>
         <v>12272727.2727273</v>
       </c>
       <c r="O6" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",D6,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A6,Huy_dong!$B$2:$B$99,"S2"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A6,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",D6,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A6,Huy_dong!$B$2:$B$100,"S2"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A6,Bang_luong!$B$2:$B$13,0))</f>
         <v>11965909.0909091</v>
       </c>
       <c r="P6" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",E6,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A6,Huy_dong!$B$2:$B$99,"S3"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A6,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",E6,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A6,Huy_dong!$B$2:$B$100,"S3"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A6,Bang_luong!$B$2:$B$13,0))</f>
         <v>14727272.7272727</v>
       </c>
       <c r="Q6" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",F6,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A6,Huy_dong!$B$2:$B$99,"S4"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A6,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",F6,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A6,Huy_dong!$B$2:$B$100,"S4"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A6,Bang_luong!$B$2:$B$13,0))</f>
         <v>9818181.81818182</v>
       </c>
       <c r="R6" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",G6,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A6,Huy_dong!$B$2:$B$99,"S5"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A6,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",G6,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A6,Huy_dong!$B$2:$B$100,"S5"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A6,Bang_luong!$B$2:$B$13,0))</f>
         <v>7363636.36363636</v>
       </c>
       <c r="S6" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",H6,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A6,Huy_dong!$B$2:$B$99,"S6"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A6,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",H6,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A6,Huy_dong!$B$2:$B$100,"S6"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A6,Bang_luong!$B$2:$B$13,0))</f>
         <v>12272727.2727273</v>
       </c>
       <c r="T6" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",I6,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A6,Huy_dong!$B$2:$B$99,"S7"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A6,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",I6,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A6,Huy_dong!$B$2:$B$100,"S7"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A6,Bang_luong!$B$2:$B$13,0))</f>
         <v>9818181.81818182</v>
       </c>
       <c r="U6" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",J6,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A6,Huy_dong!$B$2:$B$99,"S8"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A6,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",J6,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A6,Huy_dong!$B$2:$B$100,"S8"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A6,Bang_luong!$B$2:$B$13,0))</f>
         <v>4909090.90909091</v>
       </c>
       <c r="V6" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",K6,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A6,Huy_dong!$B$2:$B$99,"S9"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A6,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",K6,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A6,Huy_dong!$B$2:$B$100,"S9"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A6,Bang_luong!$B$2:$B$13,0))</f>
         <v>6750000</v>
       </c>
       <c r="W6" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",L6,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A6,Huy_dong!$B$2:$B$99,"KT"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A6,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",L6,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A6,Huy_dong!$B$2:$B$100,"KT"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A6,Bang_luong!$B$2:$B$13,0))</f>
         <v>0</v>
       </c>
       <c r="X6" s="12" t="n">
@@ -3216,43 +3216,43 @@
         <v>71.75</v>
       </c>
       <c r="N7" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",C7,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A7,Huy_dong!$B$2:$B$99,"S1"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A7,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",C7,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A7,Huy_dong!$B$2:$B$100,"S1"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A7,Bang_luong!$B$2:$B$13,0))</f>
         <v>20829545.4545455</v>
       </c>
       <c r="O7" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",D7,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A7,Huy_dong!$B$2:$B$99,"S2"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A7,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",D7,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A7,Huy_dong!$B$2:$B$100,"S2"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A7,Bang_luong!$B$2:$B$13,0))</f>
         <v>21363636.3636364</v>
       </c>
       <c r="P7" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",E7,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A7,Huy_dong!$B$2:$B$99,"S3"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A7,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",E7,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A7,Huy_dong!$B$2:$B$100,"S3"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A7,Bang_luong!$B$2:$B$13,0))</f>
         <v>25636363.6363636</v>
       </c>
       <c r="Q7" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",F7,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A7,Huy_dong!$B$2:$B$99,"S4"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A7,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",F7,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A7,Huy_dong!$B$2:$B$100,"S4"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A7,Bang_luong!$B$2:$B$13,0))</f>
         <v>21363636.3636364</v>
       </c>
       <c r="R7" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",G7,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A7,Huy_dong!$B$2:$B$99,"S5"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A7,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",G7,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A7,Huy_dong!$B$2:$B$100,"S5"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A7,Bang_luong!$B$2:$B$13,0))</f>
         <v>13886363.6363636</v>
       </c>
       <c r="S7" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",H7,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A7,Huy_dong!$B$2:$B$99,"S6"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A7,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",H7,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A7,Huy_dong!$B$2:$B$100,"S6"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A7,Bang_luong!$B$2:$B$13,0))</f>
         <v>20295454.5454545</v>
       </c>
       <c r="T7" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",I7,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A7,Huy_dong!$B$2:$B$99,"S7"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A7,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",I7,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A7,Huy_dong!$B$2:$B$100,"S7"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A7,Bang_luong!$B$2:$B$13,0))</f>
         <v>0</v>
       </c>
       <c r="U7" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",J7,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A7,Huy_dong!$B$2:$B$99,"S8"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A7,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",J7,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A7,Huy_dong!$B$2:$B$100,"S8"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A7,Bang_luong!$B$2:$B$13,0))</f>
         <v>16022727.2727273</v>
       </c>
       <c r="V7" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",K7,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A7,Huy_dong!$B$2:$B$99,"S9"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A7,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",K7,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A7,Huy_dong!$B$2:$B$100,"S9"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A7,Bang_luong!$B$2:$B$13,0))</f>
         <v>13886363.6363636</v>
       </c>
       <c r="W7" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",L7,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A7,Huy_dong!$B$2:$B$99,"KT"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A7,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",L7,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A7,Huy_dong!$B$2:$B$100,"KT"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A7,Bang_luong!$B$2:$B$13,0))</f>
         <v>0</v>
       </c>
       <c r="X7" s="12" t="n">
@@ -3312,43 +3312,43 @@
         <v>67</v>
       </c>
       <c r="N8" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",C8,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A8,Huy_dong!$B$2:$B$99,"S1"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A8,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",C8,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A8,Huy_dong!$B$2:$B$100,"S1"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A8,Bang_luong!$B$2:$B$13,0))</f>
         <v>5454545.45454545</v>
       </c>
       <c r="O8" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",D8,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A8,Huy_dong!$B$2:$B$99,"S2"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A8,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",D8,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A8,Huy_dong!$B$2:$B$100,"S2"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A8,Bang_luong!$B$2:$B$13,0))</f>
         <v>12272727.2727273</v>
       </c>
       <c r="P8" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",E8,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A8,Huy_dong!$B$2:$B$99,"S3"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A8,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",E8,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A8,Huy_dong!$B$2:$B$100,"S3"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A8,Bang_luong!$B$2:$B$13,0))</f>
         <v>12272727.2727273</v>
       </c>
       <c r="Q8" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",F8,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A8,Huy_dong!$B$2:$B$99,"S4"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A8,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",F8,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A8,Huy_dong!$B$2:$B$100,"S4"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A8,Bang_luong!$B$2:$B$13,0))</f>
         <v>12272727.2727273</v>
       </c>
       <c r="R8" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",G8,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A8,Huy_dong!$B$2:$B$99,"S5"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A8,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",G8,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A8,Huy_dong!$B$2:$B$100,"S5"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A8,Bang_luong!$B$2:$B$13,0))</f>
         <v>8863636.36363636</v>
       </c>
       <c r="S8" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",H8,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A8,Huy_dong!$B$2:$B$99,"S6"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A8,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",H8,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A8,Huy_dong!$B$2:$B$100,"S6"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A8,Bang_luong!$B$2:$B$13,0))</f>
         <v>12954545.4545455</v>
       </c>
       <c r="T8" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",I8,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A8,Huy_dong!$B$2:$B$99,"S7"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A8,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",I8,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A8,Huy_dong!$B$2:$B$100,"S7"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A8,Bang_luong!$B$2:$B$13,0))</f>
         <v>13636363.6363636</v>
       </c>
       <c r="U8" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",J8,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A8,Huy_dong!$B$2:$B$99,"S8"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A8,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",J8,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A8,Huy_dong!$B$2:$B$100,"S8"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A8,Bang_luong!$B$2:$B$13,0))</f>
         <v>2727272.72727273</v>
       </c>
       <c r="V8" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",K8,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A8,Huy_dong!$B$2:$B$99,"S9"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A8,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",K8,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A8,Huy_dong!$B$2:$B$100,"S9"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A8,Bang_luong!$B$2:$B$13,0))</f>
         <v>10909090.9090909</v>
       </c>
       <c r="W8" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",L8,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A8,Huy_dong!$B$2:$B$99,"KT"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A8,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",L8,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A8,Huy_dong!$B$2:$B$100,"KT"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A8,Bang_luong!$B$2:$B$13,0))</f>
         <v>0</v>
       </c>
       <c r="X8" s="12" t="n">
@@ -3408,43 +3408,43 @@
         <v>64.25</v>
       </c>
       <c r="N9" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",C9,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A9,Huy_dong!$B$2:$B$99,"S1"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A9,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",C9,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A9,Huy_dong!$B$2:$B$100,"S1"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A9,Bang_luong!$B$2:$B$13,0))</f>
         <v>0</v>
       </c>
       <c r="O9" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",D9,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A9,Huy_dong!$B$2:$B$99,"S2"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A9,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",D9,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A9,Huy_dong!$B$2:$B$100,"S2"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A9,Bang_luong!$B$2:$B$13,0))</f>
         <v>5454545.45454545</v>
       </c>
       <c r="P9" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",E9,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A9,Huy_dong!$B$2:$B$99,"S3"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A9,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",E9,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A9,Huy_dong!$B$2:$B$100,"S3"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A9,Bang_luong!$B$2:$B$13,0))</f>
         <v>17727272.7272727</v>
       </c>
       <c r="Q9" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",F9,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A9,Huy_dong!$B$2:$B$99,"S4"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A9,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",F9,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A9,Huy_dong!$B$2:$B$100,"S4"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A9,Bang_luong!$B$2:$B$13,0))</f>
         <v>13636363.6363636</v>
       </c>
       <c r="R9" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",G9,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A9,Huy_dong!$B$2:$B$99,"S5"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A9,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",G9,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A9,Huy_dong!$B$2:$B$100,"S5"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A9,Bang_luong!$B$2:$B$13,0))</f>
         <v>11250000</v>
       </c>
       <c r="S9" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",H9,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A9,Huy_dong!$B$2:$B$99,"S6"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A9,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",H9,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A9,Huy_dong!$B$2:$B$100,"S6"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A9,Bang_luong!$B$2:$B$13,0))</f>
         <v>6818181.81818182</v>
       </c>
       <c r="T9" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",I9,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A9,Huy_dong!$B$2:$B$99,"S7"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A9,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",I9,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A9,Huy_dong!$B$2:$B$100,"S7"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A9,Bang_luong!$B$2:$B$13,0))</f>
         <v>13636363.6363636</v>
       </c>
       <c r="U9" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",J9,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A9,Huy_dong!$B$2:$B$99,"S8"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A9,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",J9,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A9,Huy_dong!$B$2:$B$100,"S8"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A9,Bang_luong!$B$2:$B$13,0))</f>
         <v>5454545.45454545</v>
       </c>
       <c r="V9" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",K9,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A9,Huy_dong!$B$2:$B$99,"S9"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A9,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",K9,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A9,Huy_dong!$B$2:$B$100,"S9"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A9,Bang_luong!$B$2:$B$13,0))</f>
         <v>13636363.6363636</v>
       </c>
       <c r="W9" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",L9,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A9,Huy_dong!$B$2:$B$99,"KT"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A9,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",L9,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A9,Huy_dong!$B$2:$B$100,"KT"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A9,Bang_luong!$B$2:$B$13,0))</f>
         <v>0</v>
       </c>
       <c r="X9" s="12" t="n">
@@ -3504,43 +3504,43 @@
         <v>60.25</v>
       </c>
       <c r="N10" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",C10,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A10,Huy_dong!$B$2:$B$99,"S1"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A10,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",C10,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A10,Huy_dong!$B$2:$B$100,"S1"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A10,Bang_luong!$B$2:$B$13,0))</f>
         <v>4090909.09090909</v>
       </c>
       <c r="O10" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",D10,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A10,Huy_dong!$B$2:$B$99,"S2"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A10,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",D10,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A10,Huy_dong!$B$2:$B$100,"S2"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A10,Bang_luong!$B$2:$B$13,0))</f>
         <v>5454545.45454545</v>
       </c>
       <c r="P10" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",E10,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A10,Huy_dong!$B$2:$B$99,"S3"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A10,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",E10,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A10,Huy_dong!$B$2:$B$100,"S3"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A10,Bang_luong!$B$2:$B$13,0))</f>
         <v>17045454.5454545</v>
       </c>
       <c r="Q10" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",F10,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A10,Huy_dong!$B$2:$B$99,"S4"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A10,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",F10,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A10,Huy_dong!$B$2:$B$100,"S4"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A10,Bang_luong!$B$2:$B$13,0))</f>
         <v>10227272.7272727</v>
       </c>
       <c r="R10" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",G10,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A10,Huy_dong!$B$2:$B$99,"S5"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A10,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",G10,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A10,Huy_dong!$B$2:$B$100,"S5"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A10,Bang_luong!$B$2:$B$13,0))</f>
         <v>9886363.63636364</v>
       </c>
       <c r="S10" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",H10,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A10,Huy_dong!$B$2:$B$99,"S6"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A10,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",H10,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A10,Huy_dong!$B$2:$B$100,"S6"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A10,Bang_luong!$B$2:$B$13,0))</f>
         <v>8181818.18181818</v>
       </c>
       <c r="T10" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",I10,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A10,Huy_dong!$B$2:$B$99,"S7"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A10,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",I10,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A10,Huy_dong!$B$2:$B$100,"S7"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A10,Bang_luong!$B$2:$B$13,0))</f>
         <v>10909090.9090909</v>
       </c>
       <c r="U10" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",J10,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A10,Huy_dong!$B$2:$B$99,"S8"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A10,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",J10,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A10,Huy_dong!$B$2:$B$100,"S8"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A10,Bang_luong!$B$2:$B$13,0))</f>
         <v>10909090.9090909</v>
       </c>
       <c r="V10" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",K10,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A10,Huy_dong!$B$2:$B$99,"S9"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A10,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",K10,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A10,Huy_dong!$B$2:$B$100,"S9"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A10,Bang_luong!$B$2:$B$13,0))</f>
         <v>5454545.45454545</v>
       </c>
       <c r="W10" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",L10,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A10,Huy_dong!$B$2:$B$99,"KT"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A10,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",L10,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A10,Huy_dong!$B$2:$B$100,"KT"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A10,Bang_luong!$B$2:$B$13,0))</f>
         <v>0</v>
       </c>
       <c r="X10" s="12" t="n">
@@ -3600,43 +3600,43 @@
         <v>49.75</v>
       </c>
       <c r="N11" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",C11,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A11,Huy_dong!$B$2:$B$99,"S1"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A11,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",C11,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A11,Huy_dong!$B$2:$B$100,"S1"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A11,Bang_luong!$B$2:$B$13,0))</f>
         <v>0</v>
       </c>
       <c r="O11" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",D11,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A11,Huy_dong!$B$2:$B$99,"S2"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A11,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",D11,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A11,Huy_dong!$B$2:$B$100,"S2"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A11,Bang_luong!$B$2:$B$13,0))</f>
         <v>3818181.81818182</v>
       </c>
       <c r="P11" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",E11,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A11,Huy_dong!$B$2:$B$99,"S3"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A11,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",E11,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A11,Huy_dong!$B$2:$B$100,"S3"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A11,Bang_luong!$B$2:$B$13,0))</f>
         <v>10909090.9090909</v>
       </c>
       <c r="Q11" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",F11,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A11,Huy_dong!$B$2:$B$99,"S4"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A11,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",F11,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A11,Huy_dong!$B$2:$B$100,"S4"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A11,Bang_luong!$B$2:$B$13,0))</f>
         <v>10909090.9090909</v>
       </c>
       <c r="R11" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",G11,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A11,Huy_dong!$B$2:$B$99,"S5"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A11,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",G11,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A11,Huy_dong!$B$2:$B$100,"S5"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A11,Bang_luong!$B$2:$B$13,0))</f>
         <v>10090909.0909091</v>
       </c>
       <c r="S11" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",H11,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A11,Huy_dong!$B$2:$B$99,"S6"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A11,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",H11,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A11,Huy_dong!$B$2:$B$100,"S6"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A11,Bang_luong!$B$2:$B$13,0))</f>
         <v>2727272.72727273</v>
       </c>
       <c r="T11" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",I11,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A11,Huy_dong!$B$2:$B$99,"S7"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A11,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",I11,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A11,Huy_dong!$B$2:$B$100,"S7"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A11,Bang_luong!$B$2:$B$13,0))</f>
         <v>7636363.63636364</v>
       </c>
       <c r="U11" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",J11,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A11,Huy_dong!$B$2:$B$99,"S8"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A11,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",J11,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A11,Huy_dong!$B$2:$B$100,"S8"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A11,Bang_luong!$B$2:$B$13,0))</f>
         <v>2181818.18181818</v>
       </c>
       <c r="V11" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",K11,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A11,Huy_dong!$B$2:$B$99,"S9"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A11,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",K11,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A11,Huy_dong!$B$2:$B$100,"S9"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A11,Bang_luong!$B$2:$B$13,0))</f>
         <v>6000000</v>
       </c>
       <c r="W11" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",L11,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A11,Huy_dong!$B$2:$B$99,"KT"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A11,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",L11,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A11,Huy_dong!$B$2:$B$100,"KT"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A11,Bang_luong!$B$2:$B$13,0))</f>
         <v>0</v>
       </c>
       <c r="X11" s="12" t="n">
@@ -3696,43 +3696,43 @@
         <v>49.25</v>
       </c>
       <c r="N12" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",C12,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A12,Huy_dong!$B$2:$B$99,"S1"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A12,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",C12,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A12,Huy_dong!$B$2:$B$100,"S1"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A12,Bang_luong!$B$2:$B$13,0))</f>
         <v>0</v>
       </c>
       <c r="O12" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",D12,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A12,Huy_dong!$B$2:$B$99,"S2"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A12,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",D12,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A12,Huy_dong!$B$2:$B$100,"S2"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A12,Bang_luong!$B$2:$B$13,0))</f>
         <v>0</v>
       </c>
       <c r="P12" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",E12,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A12,Huy_dong!$B$2:$B$99,"S3"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A12,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",E12,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A12,Huy_dong!$B$2:$B$100,"S3"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A12,Bang_luong!$B$2:$B$13,0))</f>
         <v>6545454.54545455</v>
       </c>
       <c r="Q12" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",F12,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A12,Huy_dong!$B$2:$B$99,"S4"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A12,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",F12,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A12,Huy_dong!$B$2:$B$100,"S4"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A12,Bang_luong!$B$2:$B$13,0))</f>
         <v>9818181.81818182</v>
       </c>
       <c r="R12" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",G12,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A12,Huy_dong!$B$2:$B$99,"S5"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A12,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",G12,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A12,Huy_dong!$B$2:$B$100,"S5"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A12,Bang_luong!$B$2:$B$13,0))</f>
         <v>9000000</v>
       </c>
       <c r="S12" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",H12,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A12,Huy_dong!$B$2:$B$99,"S6"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A12,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",H12,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A12,Huy_dong!$B$2:$B$100,"S6"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A12,Bang_luong!$B$2:$B$13,0))</f>
         <v>8454545.45454545</v>
       </c>
       <c r="T12" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",I12,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A12,Huy_dong!$B$2:$B$99,"S7"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A12,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",I12,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A12,Huy_dong!$B$2:$B$100,"S7"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A12,Bang_luong!$B$2:$B$13,0))</f>
         <v>6000000</v>
       </c>
       <c r="U12" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",J12,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A12,Huy_dong!$B$2:$B$99,"S8"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A12,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",J12,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A12,Huy_dong!$B$2:$B$100,"S8"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A12,Bang_luong!$B$2:$B$13,0))</f>
         <v>5454545.45454545</v>
       </c>
       <c r="V12" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",K12,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A12,Huy_dong!$B$2:$B$99,"S9"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A12,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",K12,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A12,Huy_dong!$B$2:$B$100,"S9"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A12,Bang_luong!$B$2:$B$13,0))</f>
         <v>8454545.45454545</v>
       </c>
       <c r="W12" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",L12,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A12,Huy_dong!$B$2:$B$99,"KT"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A12,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",L12,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A12,Huy_dong!$B$2:$B$100,"KT"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A12,Bang_luong!$B$2:$B$13,0))</f>
         <v>0</v>
       </c>
       <c r="X12" s="12" t="n">
@@ -3792,43 +3792,43 @@
         <v>58.75</v>
       </c>
       <c r="N13" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",C13,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A13,Huy_dong!$B$2:$B$99,"S1"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A13,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",C13,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A13,Huy_dong!$B$2:$B$100,"S1"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A13,Bang_luong!$B$2:$B$13,0))</f>
         <v>0</v>
       </c>
       <c r="O13" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",D13,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A13,Huy_dong!$B$2:$B$99,"S2"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A13,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",D13,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A13,Huy_dong!$B$2:$B$100,"S2"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A13,Bang_luong!$B$2:$B$13,0))</f>
         <v>0</v>
       </c>
       <c r="P13" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",E13,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A13,Huy_dong!$B$2:$B$99,"S3"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A13,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",E13,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A13,Huy_dong!$B$2:$B$100,"S3"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A13,Bang_luong!$B$2:$B$13,0))</f>
         <v>17727272.7272727</v>
       </c>
       <c r="Q13" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",F13,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A13,Huy_dong!$B$2:$B$99,"S4"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A13,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",F13,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A13,Huy_dong!$B$2:$B$100,"S4"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A13,Bang_luong!$B$2:$B$13,0))</f>
         <v>12613636.3636364</v>
       </c>
       <c r="R13" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",G13,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A13,Huy_dong!$B$2:$B$99,"S5"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A13,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",G13,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A13,Huy_dong!$B$2:$B$100,"S5"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A13,Bang_luong!$B$2:$B$13,0))</f>
         <v>13636363.6363636</v>
       </c>
       <c r="S13" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",H13,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A13,Huy_dong!$B$2:$B$99,"S6"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A13,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",H13,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A13,Huy_dong!$B$2:$B$100,"S6"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A13,Bang_luong!$B$2:$B$13,0))</f>
         <v>13636363.6363636</v>
       </c>
       <c r="T13" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",I13,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A13,Huy_dong!$B$2:$B$99,"S7"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A13,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",I13,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A13,Huy_dong!$B$2:$B$100,"S7"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A13,Bang_luong!$B$2:$B$13,0))</f>
         <v>5454545.45454545</v>
       </c>
       <c r="U13" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",J13,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A13,Huy_dong!$B$2:$B$99,"S8"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A13,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",J13,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A13,Huy_dong!$B$2:$B$100,"S8"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A13,Bang_luong!$B$2:$B$13,0))</f>
         <v>6136363.63636364</v>
       </c>
       <c r="V13" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",K13,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A13,Huy_dong!$B$2:$B$99,"S9"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A13,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",K13,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A13,Huy_dong!$B$2:$B$100,"S9"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A13,Bang_luong!$B$2:$B$13,0))</f>
         <v>10909090.9090909</v>
       </c>
       <c r="W13" s="12" t="n">
-        <f aca="false">IF(Tham_so!$B$11="cong_suc",L13,SUMIFS(Huy_dong!$C$2:$C$99,Huy_dong!$A$2:$A$99,$A13,Huy_dong!$B$2:$B$99,"KT"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A13,Bang_luong!$B$2:$B$13,0))</f>
+        <f aca="false">IF(Tham_so!$B$11="cong_suc",L13,SUMIFS(Huy_dong!$C$2:$C$100,Huy_dong!$A$2:$A$100,$A13,Huy_dong!$B$2:$B$100,"KT"))*INDEX(Bang_luong!$L$2:$L$13,MATCH($A13,Bang_luong!$B$2:$B$13,0))</f>
         <v>0</v>
       </c>
       <c r="X13" s="12" t="n">
@@ -4002,7 +4002,7 @@
       </c>
       <c r="B5" s="8" t="n">
         <f aca="false">Bang_luong!G14</f>
-        <v>908</v>
+        <v>921</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>102</v>
@@ -4024,7 +4024,7 @@
       </c>
       <c r="B7" s="8" t="n">
         <f aca="false">Bang_luong!I14</f>
-        <v>171.25</v>
+        <v>184.25</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>104</v>
@@ -4036,7 +4036,7 @@
       </c>
       <c r="B8" s="19" t="n">
         <f aca="false">IF(B5=0,0,B6/B5)</f>
-        <v>0.811398678414097</v>
+        <v>0.799945711183496</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>106</v>
@@ -23265,7 +23265,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C101"/>
+  <dimension ref="A1:C102"/>
   <sheetFormatPr defaultColWidth="8.515625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -23465,21 +23465,21 @@
         <v>41</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>6</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="C19" s="7" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23487,7 +23487,7 @@
         <v>44</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C20" s="7" t="n">
         <v>10</v>
@@ -23498,10 +23498,10 @@
         <v>44</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C21" s="7" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23509,10 +23509,10 @@
         <v>44</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C22" s="7" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23520,7 +23520,7 @@
         <v>44</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C23" s="7" t="n">
         <v>10</v>
@@ -23531,7 +23531,7 @@
         <v>44</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C24" s="7" t="n">
         <v>10</v>
@@ -23542,10 +23542,10 @@
         <v>44</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C25" s="7" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23553,21 +23553,21 @@
         <v>44</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C26" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="C27" s="7" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23575,7 +23575,7 @@
         <v>47</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C28" s="7" t="n">
         <v>10</v>
@@ -23586,10 +23586,10 @@
         <v>47</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C29" s="7" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23597,10 +23597,10 @@
         <v>47</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C30" s="7" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23608,7 +23608,7 @@
         <v>47</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C31" s="7" t="n">
         <v>10</v>
@@ -23619,7 +23619,7 @@
         <v>47</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C32" s="7" t="n">
         <v>10</v>
@@ -23630,10 +23630,10 @@
         <v>47</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C33" s="7" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23641,18 +23641,18 @@
         <v>47</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C34" s="7" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="C35" s="7" t="n">
         <v>10</v>
@@ -23663,7 +23663,7 @@
         <v>49</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C36" s="7" t="n">
         <v>10</v>
@@ -23674,10 +23674,10 @@
         <v>49</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C37" s="7" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23685,10 +23685,10 @@
         <v>49</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C38" s="7" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23696,7 +23696,7 @@
         <v>49</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C39" s="7" t="n">
         <v>10</v>
@@ -23707,7 +23707,7 @@
         <v>49</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C40" s="7" t="n">
         <v>10</v>
@@ -23718,10 +23718,10 @@
         <v>49</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C41" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23729,10 +23729,10 @@
         <v>49</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C42" s="7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23740,21 +23740,21 @@
         <v>49</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C43" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="6" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="C44" s="7" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23762,7 +23762,7 @@
         <v>52</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C45" s="7" t="n">
         <v>10</v>
@@ -23773,10 +23773,10 @@
         <v>52</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C46" s="7" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23784,10 +23784,10 @@
         <v>52</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C47" s="7" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23795,7 +23795,7 @@
         <v>52</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C48" s="7" t="n">
         <v>10</v>
@@ -23806,7 +23806,7 @@
         <v>52</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C49" s="7" t="n">
         <v>10</v>
@@ -23817,10 +23817,10 @@
         <v>52</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C50" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23828,21 +23828,21 @@
         <v>52</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C51" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="6" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="C52" s="7" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23850,7 +23850,7 @@
         <v>56</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C53" s="7" t="n">
         <v>10</v>
@@ -23861,10 +23861,10 @@
         <v>56</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C54" s="7" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23872,10 +23872,10 @@
         <v>56</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C55" s="7" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23883,7 +23883,7 @@
         <v>56</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C56" s="7" t="n">
         <v>10</v>
@@ -23894,7 +23894,7 @@
         <v>56</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C57" s="7" t="n">
         <v>10</v>
@@ -23905,7 +23905,7 @@
         <v>56</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C58" s="7" t="n">
         <v>10</v>
@@ -23916,10 +23916,10 @@
         <v>56</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C59" s="7" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23927,21 +23927,21 @@
         <v>56</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C60" s="7" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="6" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="C61" s="7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23949,10 +23949,10 @@
         <v>58</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23960,10 +23960,10 @@
         <v>58</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C63" s="7" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23971,7 +23971,7 @@
         <v>58</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C64" s="7" t="n">
         <v>10</v>
@@ -23982,7 +23982,7 @@
         <v>58</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C65" s="7" t="n">
         <v>10</v>
@@ -23993,7 +23993,7 @@
         <v>58</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C66" s="7" t="n">
         <v>10</v>
@@ -24004,10 +24004,10 @@
         <v>58</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C67" s="7" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24015,18 +24015,18 @@
         <v>58</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="6" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="C69" s="7" t="n">
         <v>10</v>
@@ -24037,7 +24037,7 @@
         <v>60</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C70" s="7" t="n">
         <v>10</v>
@@ -24048,10 +24048,10 @@
         <v>60</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C71" s="7" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24059,10 +24059,10 @@
         <v>60</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24070,7 +24070,7 @@
         <v>60</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C73" s="7" t="n">
         <v>10</v>
@@ -24081,7 +24081,7 @@
         <v>60</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C74" s="7" t="n">
         <v>10</v>
@@ -24092,7 +24092,7 @@
         <v>60</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C75" s="7" t="n">
         <v>10</v>
@@ -24103,10 +24103,10 @@
         <v>60</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C76" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24114,21 +24114,21 @@
         <v>60</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C77" s="7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B78" s="6" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="C78" s="7" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24136,10 +24136,10 @@
         <v>62</v>
       </c>
       <c r="B79" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C79" s="7" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24147,10 +24147,10 @@
         <v>62</v>
       </c>
       <c r="B80" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C80" s="7" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24158,7 +24158,7 @@
         <v>62</v>
       </c>
       <c r="B81" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C81" s="7" t="n">
         <v>10</v>
@@ -24169,7 +24169,7 @@
         <v>62</v>
       </c>
       <c r="B82" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C82" s="7" t="n">
         <v>10</v>
@@ -24180,10 +24180,10 @@
         <v>62</v>
       </c>
       <c r="B83" s="6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C83" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24191,10 +24191,10 @@
         <v>62</v>
       </c>
       <c r="B84" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C84" s="7" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24202,21 +24202,21 @@
         <v>62</v>
       </c>
       <c r="B85" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C85" s="7" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="6" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B86" s="6" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="C86" s="7" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24224,10 +24224,10 @@
         <v>65</v>
       </c>
       <c r="B87" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C87" s="7" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24235,7 +24235,7 @@
         <v>65</v>
       </c>
       <c r="B88" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C88" s="7" t="n">
         <v>10</v>
@@ -24246,7 +24246,7 @@
         <v>65</v>
       </c>
       <c r="B89" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C89" s="7" t="n">
         <v>10</v>
@@ -24257,10 +24257,10 @@
         <v>65</v>
       </c>
       <c r="B90" s="6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C90" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24268,10 +24268,10 @@
         <v>65</v>
       </c>
       <c r="B91" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C91" s="7" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24279,21 +24279,21 @@
         <v>65</v>
       </c>
       <c r="B92" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C92" s="7" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="6" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B93" s="6" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="C93" s="7" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24301,10 +24301,10 @@
         <v>67</v>
       </c>
       <c r="B94" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C94" s="7" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24312,7 +24312,7 @@
         <v>67</v>
       </c>
       <c r="B95" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C95" s="7" t="n">
         <v>10</v>
@@ -24323,7 +24323,7 @@
         <v>67</v>
       </c>
       <c r="B96" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C96" s="7" t="n">
         <v>10</v>
@@ -24334,10 +24334,10 @@
         <v>67</v>
       </c>
       <c r="B97" s="6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C97" s="7" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24345,10 +24345,10 @@
         <v>67</v>
       </c>
       <c r="B98" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C98" s="7" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24356,14 +24356,25 @@
         <v>67</v>
       </c>
       <c r="B99" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="C99" s="7" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B100" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="C99" s="7" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="17" t="s">
+      <c r="C100" s="7" t="n">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="17" t="s">
         <v>321</v>
       </c>
     </row>

</xml_diff>